<commit_message>
Diamond lead run: round-5 LinkedIn workbook, people workbook, compiled refresh
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-16T10:11:18+00:00</t>
+          <t>2026-10-16T10:40:04+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-6 partial merge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-16T10:40:04+00:00</t>
+          <t>2026-10-16T18:07:16+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-6 merged, round-6 workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-16T18:07:16+00:00</t>
+          <t>2026-10-16T18:35:30+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-7 partial merge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-16T18:35:30+00:00</t>
+          <t>2026-10-16T19:09:18+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-7 complete, round-7 workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-16T19:09:18+00:00</t>
+          <t>2026-10-16T19:36:04+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-8 complete, round-8 workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:07+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-16T19:36:04+00:00</t>
+          <t>2026-10-17T05:29:08+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-9 (50 cities) complete, round-9 workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:07+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-17T05:29:08+00:00</t>
+          <t>2026-10-17T06:39:17+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-10 qualify-push partial merge (285 -> 425 qualified)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-17T06:39:17+00:00</t>
+          <t>2026-10-18T11:45:35+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-10 qualify-push merge #2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-18T11:45:35+00:00</t>
+          <t>2026-10-18T12:19:21+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-11 qualify-push merge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-18T12:19:21+00:00</t>
+          <t>2026-10-19T14:02:04+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-11 qualify-push complete, round-11 workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-19T14:02:04+00:00</t>
+          <t>2026-10-19T14:34:59+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-12 qualify-push merge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-19T14:34:59+00:00</t>
+          <t>2026-10-19T20:33:31+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diamond lead run: round-12 qualify-push complete, round-12 workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YvEgMG8dQ2X5nK4MYwD7D
</commit_message>
<xml_diff>
--- a/leadrun_diamonds/diamond_leads_people.xlsx
+++ b/leadrun_diamonds/diamond_leads_people.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8390,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11652,7 +11652,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13864,7 +13864,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14440,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15500,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15565,7 +15565,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16121,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16450,7 +16450,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17229,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17302,7 +17302,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17424,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17712,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17850,7 +17850,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18154,7 +18154,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18381,7 +18381,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18531,7 +18531,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18831,7 +18831,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19265,7 +19265,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19330,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19695,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19837,7 +19837,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20210,7 +20210,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20283,7 +20283,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20429,7 +20429,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20652,7 +20652,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21025,7 +21025,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21094,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21601,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -21974,7 +21974,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-19T20:33:31+00:00</t>
+          <t>2026-10-19T20:57:45+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>